<commit_message>
simulation speed toggle, general UI improvements
</commit_message>
<xml_diff>
--- a/1.7.26 Hatherly, Luke - NEA Marking Grid.xlsx
+++ b/1.7.26 Hatherly, Luke - NEA Marking Grid.xlsx
@@ -7273,8 +7273,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100878E5A16D2E5BD44B76BEF7FA841D917" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="416d995b46902b136ce492dff88067f5">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ee41aa2-a9ad-41d9-b8b1-bb01358df394" xmlns:ns3="cc0e8f53-4a54-4e8b-83c1-d15ba22c3663" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1396db6f1b8939c432c538e4a6e33256" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100878E5A16D2E5BD44B76BEF7FA841D917" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8cfd750772889e51922bf98afcd7fef6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ee41aa2-a9ad-41d9-b8b1-bb01358df394" xmlns:ns3="cc0e8f53-4a54-4e8b-83c1-d15ba22c3663" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="be8fb80e2decf39920ea00b104793a28" ns2:_="" ns3:_="">
     <xsd:import namespace="7ee41aa2-a9ad-41d9-b8b1-bb01358df394"/>
     <xsd:import namespace="cc0e8f53-4a54-4e8b-83c1-d15ba22c3663"/>
     <xsd:element name="properties">
@@ -7292,6 +7292,7 @@
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -7344,6 +7345,11 @@
     <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -7481,20 +7487,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{964298F4-DCF9-4AF6-849B-C2D77A8115EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7ee41aa2-a9ad-41d9-b8b1-bb01358df394"/>
-    <ds:schemaRef ds:uri="cc0e8f53-4a54-4e8b-83c1-d15ba22c3663"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8384F50E-FF87-4239-B5DE-CB6621A06C7B}"/>
 </file>
</xml_diff>